<commit_message>
converted code to functions
</commit_message>
<xml_diff>
--- a/notebooks/3_spatiotemporal/2_correlation_mugging_tone.xlsx
+++ b/notebooks/3_spatiotemporal/2_correlation_mugging_tone.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://olddominion-my.sharepoint.com/personal/jmart130_odu_edu/Documents/GITHUB_VMASC/twitter_analysis_col/notebooks/3_spatiotemporal/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="8_{F51FD362-AD1C-3645-B1D4-51955FCCDF5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1EE09878-4728-9D46-B0C0-DFA1FC0DA433}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="8_{F51FD362-AD1C-3645-B1D4-51955FCCDF5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B80AFEC-C292-E44D-BEC5-89742C19E138}"/>
   <bookViews>
     <workbookView xWindow="3880" yWindow="3060" windowWidth="27240" windowHeight="16440" xr2:uid="{CE39F28C-9F2E-284D-9972-358C8C26C2AA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -220,6 +220,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1216,7 +1220,7 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F2:F33">
+  <conditionalFormatting sqref="D2:D33">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -1228,7 +1232,31 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D33">
+  <conditionalFormatting sqref="F2:F33">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C2:C33">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2:B33">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>